<commit_message>
feat(finance): Registro Corrispettivi commercialista F1+F2 e riclassifica DC Studio
Aliquota unica 10% su corrispettivi, export F1+F2 con controlli bloccanti, API/UI primaria e privacy in prebuild. F3 sospeso. Bonifico DC Studio riclassificato CONSULENZE; audit bonifico→fiorista 2026 in sola lettura.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/verbali/FloreMoria_2026_T2_Corrispettivi.xlsx
+++ b/docs/verbali/FloreMoria_2026_T2_Corrispettivi.xlsx
@@ -6,14 +6,13 @@
   <sheets>
     <sheet sheetId="1" name="F1 — Riepilogo" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="F2 — Registro corrispettivi" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="F3 — Costi senza documento" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="33">
   <si>
     <t>Ragione sociale</t>
   </si>
@@ -36,7 +35,7 @@
     <t>Data e ora generazione</t>
   </si>
   <si>
-    <t>20/09/2026, 15:15:20</t>
+    <t>20/09/2026, 19:23:45</t>
   </si>
   <si>
     <t>Voce</t>
@@ -60,18 +59,12 @@
     <t>Vendite IVA 10%</t>
   </si>
   <si>
-    <t>Vendite IVA 22%</t>
-  </si>
-  <si>
-    <t>Aliquota mancante</t>
+    <t>TOTALE</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>TOTALE</t>
-  </si>
-  <si>
     <t>Nota 1</t>
   </si>
   <si>
@@ -81,7 +74,19 @@
     <t>Nota 2</t>
   </si>
   <si>
-    <t>Per i costi fiorista senza fattura/scontrino nel periodo vedere il foglio «F3 — Costi senza documento».</t>
+    <t>Aliquota unica 10% su tutto il corrispettivo (accessorietà — METODO §8.3).</t>
+  </si>
+  <si>
+    <t>Nota 3</t>
+  </si>
+  <si>
+    <t>Foglio F3 (costi fiorista senza documento) sospeso: rientrerà quando l’abbinamento bonifici→consegne sarà corretto. Non usare i movimenti bancari come proxy del costo per consegna.</t>
+  </si>
+  <si>
+    <t>Nota 4</t>
+  </si>
+  <si>
+    <t>Prima di chiudere il trimestre caricare l’estratto conto Fineco aggiornato in Contabilità → Movimenti bancari.</t>
   </si>
   <si>
     <t>Data ordine</t>
@@ -96,6 +101,9 @@
     <t>IVA EUR</t>
   </si>
   <si>
+    <t>DA_COLLEGARE</t>
+  </si>
+  <si>
     <t>Stripe</t>
   </si>
   <si>
@@ -103,66 +111,6 @@
   </si>
   <si>
     <t>FT-MC-26-007</t>
-  </si>
-  <si>
-    <t>Fiorista</t>
-  </si>
-  <si>
-    <t>Importo EUR</t>
-  </si>
-  <si>
-    <t>Data consegna</t>
-  </si>
-  <si>
-    <t>cmtvn3gt00</t>
-  </si>
-  <si>
-    <t>SHOPPINGARDEN di Anna Bruno</t>
-  </si>
-  <si>
-    <t>Mastro Fiori</t>
-  </si>
-  <si>
-    <t>Carrozza</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>Fioreria Reggio Calabria</t>
-  </si>
-  <si>
-    <t>Fioreria Battistella s.r.l.</t>
-  </si>
-  <si>
-    <t>Davide Capitano</t>
-  </si>
-  <si>
-    <t>Calamunci Tindaro</t>
-  </si>
-  <si>
-    <t>Cingolani Antonella</t>
-  </si>
-  <si>
-    <t>FT-SA-26-002</t>
-  </si>
-  <si>
-    <t>Floragarden di Stinga Baldassarre</t>
-  </si>
-  <si>
-    <t>FT-PA-26-003</t>
-  </si>
-  <si>
-    <t>FT-CS-26-001</t>
-  </si>
-  <si>
-    <t>FT-RC-26-001</t>
-  </si>
-  <si>
-    <t>FT-PA-26-004</t>
-  </si>
-  <si>
-    <t>FT-CS-26-002</t>
   </si>
 </sst>
 </file>
@@ -655,96 +603,72 @@
         <v>14</v>
       </c>
       <c r="B7" s="2">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C7" s="3">
-        <v>786.14</v>
+        <v>1132.73</v>
       </c>
       <c r="D7" s="2">
         <v>10</v>
       </c>
       <c r="E7" s="3">
-        <v>78.63</v>
+        <v>113.29</v>
       </c>
       <c r="F7" s="3">
-        <v>864.77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+        <v>1246.02</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="2">
-        <v>5</v>
-      </c>
-      <c r="C8" s="3">
-        <v>40.1</v>
-      </c>
-      <c r="D8" s="2">
+      <c r="B8" s="5">
         <v>22</v>
       </c>
-      <c r="E8" s="3">
-        <v>8.82</v>
-      </c>
-      <c r="F8" s="3">
-        <v>48.92</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="C8" s="6">
+        <v>1132.73</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2">
-        <v>9</v>
-      </c>
-      <c r="C9" s="3">
-        <v>0</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="E8" s="6">
+        <v>113.29</v>
+      </c>
+      <c r="F8" s="6">
+        <v>1246.02</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="3">
-        <v>0</v>
-      </c>
-      <c r="F9" s="3">
-        <v>332.33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="B10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="5">
-        <v>27</v>
-      </c>
-      <c r="C10" s="6">
-        <v>826.24</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="6">
-        <v>87.45</v>
-      </c>
-      <c r="F10" s="6">
-        <v>1246.02</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -755,7 +679,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -768,13 +692,13 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>10</v>
@@ -783,7 +707,7 @@
         <v>11</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>13</v>
@@ -794,10 +718,10 @@
         <v>46113.41666666667</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D2" s="3">
         <v>27.26</v>
@@ -817,10 +741,10 @@
         <v>46128.41666666667</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D3" s="3">
         <v>27.26</v>
@@ -840,10 +764,10 @@
         <v>46132.41666666667</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D4" s="3">
         <v>36.35</v>
@@ -863,10 +787,10 @@
         <v>46132.41666666667</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D5" s="3">
         <v>54.53</v>
@@ -886,10 +810,10 @@
         <v>46139.41666666667</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D6" s="3">
         <v>36.35</v>
@@ -909,125 +833,125 @@
         <v>46140.41666666667</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D7" s="3">
-        <v>12.29</v>
+        <v>49.98</v>
       </c>
       <c r="E7" s="2">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F7" s="3">
-        <v>2.7</v>
+        <v>5</v>
       </c>
       <c r="G7" s="3">
-        <v>14.99</v>
+        <v>54.98</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46140.41666666667</v>
+        <v>46141.41666666667</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D8" s="3">
-        <v>36.35</v>
+        <v>41.79</v>
       </c>
       <c r="E8" s="2">
         <v>10</v>
       </c>
       <c r="F8" s="3">
-        <v>3.64</v>
+        <v>4.18</v>
       </c>
       <c r="G8" s="3">
-        <v>39.99</v>
+        <v>45.97</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
-        <v>46141.41666666667</v>
+        <v>46145.41666666667</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D9" s="3">
-        <v>36.35</v>
+        <v>48.62</v>
       </c>
       <c r="E9" s="2">
         <v>10</v>
       </c>
       <c r="F9" s="3">
-        <v>3.64</v>
+        <v>4.86</v>
       </c>
       <c r="G9" s="3">
-        <v>39.99</v>
+        <v>53.48</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46141.41666666667</v>
+        <v>46145.41666666667</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D10" s="3">
-        <v>4.9</v>
+        <v>259</v>
       </c>
       <c r="E10" s="2">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F10" s="3">
-        <v>1.08</v>
+        <v>25.9</v>
       </c>
       <c r="G10" s="3">
-        <v>5.98</v>
+        <v>284.9</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
-        <v>46145.41666666667</v>
+        <v>46153.41666666667</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D11" s="3">
-        <v>2.86</v>
+        <v>27.26</v>
       </c>
       <c r="E11" s="2">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F11" s="3">
-        <v>0.63</v>
+        <v>2.73</v>
       </c>
       <c r="G11" s="3">
-        <v>3.49</v>
+        <v>29.99</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46145.41666666667</v>
+        <v>46158.41666666667</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D12" s="3">
         <v>45.45</v>
@@ -1044,718 +968,278 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
-        <v>46145.41666666667</v>
+        <v>46161.41666666667</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D13" s="3">
-        <v>259</v>
+        <v>31.81</v>
       </c>
       <c r="E13" s="2">
         <v>10</v>
       </c>
       <c r="F13" s="3">
-        <v>25.9</v>
+        <v>3.18</v>
       </c>
       <c r="G13" s="3">
-        <v>284.9</v>
+        <v>34.99</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="7">
-        <v>46153.41666666667</v>
+        <v>46162.41666666667</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>17</v>
+        <v>30</v>
+      </c>
+      <c r="D14" s="3">
+        <v>28.62</v>
+      </c>
+      <c r="E14" s="2">
+        <v>10</v>
+      </c>
+      <c r="F14" s="3">
+        <v>2.86</v>
       </c>
       <c r="G14" s="3">
-        <v>29.99</v>
+        <v>31.48</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
-        <v>46158.41666666667</v>
+        <v>46162.41666666667</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D15" s="3">
-        <v>45.45</v>
+        <v>28.62</v>
       </c>
       <c r="E15" s="2">
         <v>10</v>
       </c>
       <c r="F15" s="3">
-        <v>4.54</v>
+        <v>2.86</v>
       </c>
       <c r="G15" s="3">
-        <v>49.99</v>
+        <v>31.48</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="7">
-        <v>46161.41666666667</v>
+        <v>46165.41666666667</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>17</v>
+        <v>31</v>
+      </c>
+      <c r="D16" s="3">
+        <v>29.53</v>
+      </c>
+      <c r="E16" s="2">
+        <v>10</v>
+      </c>
+      <c r="F16" s="3">
+        <v>2.95</v>
       </c>
       <c r="G16" s="3">
-        <v>34.99</v>
+        <v>32.48</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46162.41666666667</v>
+        <v>46167.41666666667</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>17</v>
+        <v>30</v>
+      </c>
+      <c r="D17" s="3">
+        <v>77.25</v>
+      </c>
+      <c r="E17" s="2">
+        <v>10</v>
+      </c>
+      <c r="F17" s="3">
+        <v>7.73</v>
       </c>
       <c r="G17" s="3">
-        <v>31.48</v>
+        <v>84.98</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="7">
-        <v>46162.41666666667</v>
+        <v>46178.41666666667</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>17</v>
+        <v>30</v>
+      </c>
+      <c r="D18" s="3">
+        <v>81.81</v>
+      </c>
+      <c r="E18" s="2">
+        <v>10</v>
+      </c>
+      <c r="F18" s="3">
+        <v>8.18</v>
       </c>
       <c r="G18" s="3">
-        <v>31.48</v>
+        <v>89.99</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="7">
-        <v>46165.41666666667</v>
+        <v>46186.41666666667</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>17</v>
+        <v>30</v>
+      </c>
+      <c r="D19" s="3">
+        <v>39.97</v>
+      </c>
+      <c r="E19" s="2">
+        <v>10</v>
+      </c>
+      <c r="F19" s="3">
+        <v>4</v>
       </c>
       <c r="G19" s="3">
-        <v>32.48</v>
+        <v>43.97</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="7">
-        <v>46167.41666666667</v>
+        <v>46189.41666666667</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D20" s="3">
-        <v>63.63</v>
+        <v>44.96</v>
       </c>
       <c r="E20" s="2">
         <v>10</v>
       </c>
       <c r="F20" s="3">
-        <v>6.36</v>
+        <v>4.5</v>
       </c>
       <c r="G20" s="3">
-        <v>69.99</v>
+        <v>49.46</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="7">
-        <v>46167.41666666667</v>
+        <v>46190.41666666667</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D21" s="3">
-        <v>12.29</v>
+        <v>28.62</v>
       </c>
       <c r="E21" s="2">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F21" s="3">
-        <v>2.7</v>
+        <v>2.86</v>
       </c>
       <c r="G21" s="3">
-        <v>14.99</v>
+        <v>31.48</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46178.41666666667</v>
+        <v>46190.41666666667</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D22" s="3">
-        <v>81.81</v>
+        <v>28.62</v>
       </c>
       <c r="E22" s="2">
         <v>10</v>
       </c>
       <c r="F22" s="3">
-        <v>8.18</v>
+        <v>2.86</v>
       </c>
       <c r="G22" s="3">
-        <v>89.99</v>
+        <v>31.48</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="7">
-        <v>46186.41666666667</v>
+        <v>46195.41666666667</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>17</v>
+        <v>30</v>
+      </c>
+      <c r="D23" s="3">
+        <v>59.07</v>
+      </c>
+      <c r="E23" s="2">
+        <v>10</v>
+      </c>
+      <c r="F23" s="3">
+        <v>5.91</v>
       </c>
       <c r="G23" s="3">
-        <v>43.97</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="7">
-        <v>46189.41666666667</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" s="3">
-        <v>36.35</v>
-      </c>
-      <c r="E24" s="2">
-        <v>10</v>
-      </c>
-      <c r="F24" s="3">
-        <v>3.64</v>
-      </c>
-      <c r="G24" s="3">
-        <v>39.99</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="7">
-        <v>46189.41666666667</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" s="3">
-        <v>7.76</v>
-      </c>
-      <c r="E25" s="2">
-        <v>22</v>
-      </c>
-      <c r="F25" s="3">
-        <v>1.71</v>
-      </c>
-      <c r="G25" s="3">
-        <v>9.47</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="7">
-        <v>46190.41666666667</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G26" s="3">
-        <v>31.48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="7">
-        <v>46190.41666666667</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G27" s="3">
-        <v>31.48</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="7">
-        <v>46195.41666666667</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G28" s="3">
         <v>64.98</v>
       </c>
     </row>
-    <row r="29" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" s="6">
-        <v>826.24</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F29" s="6">
-        <v>87.45</v>
-      </c>
-      <c r="G29" s="6">
+    <row r="24" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="6">
+        <v>1132.73</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="6">
+        <v>113.29</v>
+      </c>
+      <c r="G24" s="6">
         <v>1246.02</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="35" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" s="3">
-        <v>20</v>
-      </c>
-      <c r="D2" s="7">
-        <v>46113.41666666667</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="3">
-        <v>20</v>
-      </c>
-      <c r="D3" s="7">
-        <v>46113.41666666667</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="3">
-        <v>20</v>
-      </c>
-      <c r="D4" s="7">
-        <v>46113.41666666667</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="3">
-        <v>20</v>
-      </c>
-      <c r="D5" s="7">
-        <v>46113.41666666667</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="3">
-        <v>25</v>
-      </c>
-      <c r="D6" s="7">
-        <v>46116.41666666667</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="3">
-        <v>145</v>
-      </c>
-      <c r="D7" s="7">
-        <v>46119.41666666667</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="3">
-        <v>25</v>
-      </c>
-      <c r="D8" s="7">
-        <v>46132.41666666667</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="3">
-        <v>18</v>
-      </c>
-      <c r="D9" s="7">
-        <v>46134.41666666667</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="3">
-        <v>25</v>
-      </c>
-      <c r="D10" s="7">
-        <v>46144.41666666667</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="3">
-        <v>20</v>
-      </c>
-      <c r="D11" s="7">
-        <v>46145.41666666667</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="3">
-        <v>20</v>
-      </c>
-      <c r="D12" s="7">
-        <v>46145.41666666667</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="3">
-        <v>500</v>
-      </c>
-      <c r="D13" s="7">
-        <v>46164.41666666667</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="3">
-        <v>18</v>
-      </c>
-      <c r="D14" s="7">
-        <v>46164.41666666667</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="3">
-        <v>20</v>
-      </c>
-      <c r="D15" s="7">
-        <v>46164.41666666667</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" s="3">
-        <v>40</v>
-      </c>
-      <c r="D16" s="7">
-        <v>46168.41666666667</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" s="3">
-        <v>40</v>
-      </c>
-      <c r="D17" s="7">
-        <v>46173.41666666667</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="3">
-        <v>25</v>
-      </c>
-      <c r="D18" s="7">
-        <v>46188.41666666667</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C19" s="3">
-        <v>30</v>
-      </c>
-      <c r="D19" s="7">
-        <v>46189.41666666667</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="3">
-        <v>18</v>
-      </c>
-      <c r="D20" s="7">
-        <v>46192.41666666667</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="3">
-        <v>20</v>
-      </c>
-      <c r="D21" s="7">
-        <v>46192.41666666667</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="6">
-        <v>1069</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>